<commit_message>
added issue tracking for individual missing units
</commit_message>
<xml_diff>
--- a/src/dbimporter/data/baddata.xlsx
+++ b/src/dbimporter/data/baddata.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -177,8 +177,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -200,62 +204,60 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="H2" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="0" t="s">
+      <c r="B3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -276,27 +278,27 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -317,66 +319,66 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>